<commit_message>
Implement offline-first localStorage caching, direct UI rendering, disable browser API caching, and fix bat file line endings
</commit_message>
<xml_diff>
--- a/Controle_de_Horas_Trabalho-1.xlsx
+++ b/Controle_de_Horas_Trabalho-1.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="260">
   <si>
     <t>Data</t>
   </si>
@@ -158,6 +158,36 @@
   </si>
   <si>
     <t>08:24</t>
+  </si>
+  <si>
+    <t>08:15</t>
+  </si>
+  <si>
+    <t>12:15</t>
+  </si>
+  <si>
+    <t>13:15</t>
+  </si>
+  <si>
+    <t>17:15</t>
+  </si>
+  <si>
+    <t>Teste API</t>
+  </si>
+  <si>
+    <t>Pendente</t>
+  </si>
+  <si>
+    <t>07:15</t>
+  </si>
+  <si>
+    <t>17:45</t>
+  </si>
+  <si>
+    <t>01:30</t>
+  </si>
+  <si>
+    <t>10:30</t>
   </si>
   <si>
     <t>Soma de Valor do Dia (R$)</t>
@@ -5147,7 +5177,7 @@
         <v>127.4</v>
       </c>
     </row>
-    <row r="152" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="152" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="6">
         <v>46173</v>
       </c>
@@ -5203,20 +5233,52 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="155" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A155" s="6">
         <v>46176</v>
       </c>
       <c r="B155" t="s">
         <v>24</v>
       </c>
+      <c r="C155" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D155" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E155" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F155" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="G155" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H155" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>96</v>
+      </c>
+      <c r="I155">
+        <v>12</v>
+      </c>
+      <c r="J155" t="s">
+        <v>51</v>
+      </c>
+      <c r="K155" t="s">
+        <v>52</v>
+      </c>
+      <c r="L155" t="s">
+        <v>53</v>
+      </c>
+      <c r="M155" t="s">
+        <v>54</v>
+      </c>
+      <c r="N155" t="s">
+        <v>55</v>
+      </c>
+      <c r="O155" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="156" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9312,22 +9374,22 @@
   <sheetData>
     <row r="1" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -9343,1549 +9405,1549 @@
   <sheetData>
     <row r="1" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="B2" s="22">
         <v>46028</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D2">
         <v>9.8</v>
       </c>
       <c r="E2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="B3" s="22">
         <v>46029</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="D3">
         <v>12.4</v>
       </c>
       <c r="E3" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B4" s="22">
         <v>46030</v>
       </c>
       <c r="C4" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="D4">
         <v>10.4</v>
       </c>
       <c r="E4" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B5" s="22">
         <v>46031</v>
       </c>
       <c r="C5" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="D5">
         <v>9.4</v>
       </c>
       <c r="E5" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B6" s="22">
         <v>46032</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="D6">
         <v>26.200000000000003</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B7" s="22">
         <v>46035</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="D7">
         <v>9.4</v>
       </c>
       <c r="E7" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="B8" s="22">
         <v>46036</v>
       </c>
       <c r="C8" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="D8">
         <v>9.600000000000001</v>
       </c>
       <c r="E8" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="B9" s="22">
         <v>46037</v>
       </c>
       <c r="C9" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="D9">
         <v>11.8</v>
       </c>
       <c r="E9" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B10" s="22">
         <v>46038</v>
       </c>
       <c r="C10" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="D10">
         <v>10.200000000000001</v>
       </c>
       <c r="E10" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="B11" s="22">
         <v>46039</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="D11">
         <v>24.32</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="B12" s="22">
         <v>46042</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="D12">
         <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="B13" s="22">
         <v>46043</v>
       </c>
       <c r="C13" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="D13">
         <v>11.8</v>
       </c>
       <c r="E13" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="B14" s="22">
         <v>46044</v>
       </c>
       <c r="C14" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="D14">
         <v>9.4</v>
       </c>
       <c r="E14" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="B15" s="22">
         <v>46045</v>
       </c>
       <c r="C15" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="D15">
         <v>10.200000000000001</v>
       </c>
       <c r="E15" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="B16" s="22">
         <v>46046</v>
       </c>
       <c r="C16" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="D16">
         <v>18.6</v>
       </c>
       <c r="E16" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="B17" s="22">
         <v>46049</v>
       </c>
       <c r="C17" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D17">
         <v>16.6</v>
       </c>
       <c r="E17" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="B18" s="22">
         <v>46050</v>
       </c>
       <c r="C18" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="D18">
         <v>11.200000000000001</v>
       </c>
       <c r="E18" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="B19" s="22">
         <v>46051</v>
       </c>
       <c r="C19" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="D19">
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="B20" s="22">
         <v>46052</v>
       </c>
       <c r="C20" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="D20">
         <v>11.280000000000001</v>
       </c>
       <c r="E20" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B21" s="22">
         <v>46053</v>
       </c>
       <c r="C21" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="D21">
         <v>24</v>
       </c>
       <c r="E21" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="B22" s="22">
         <v>46057</v>
       </c>
       <c r="C22" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="D22">
         <v>8.6</v>
       </c>
       <c r="E22" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="B23" s="22">
         <v>46058</v>
       </c>
       <c r="C23" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="D23">
         <v>9.4</v>
       </c>
       <c r="E23" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="B24" s="22">
         <v>46059</v>
       </c>
       <c r="C24" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="D24">
         <v>10.200000000000001</v>
       </c>
       <c r="E24" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="B25" s="22">
         <v>46060</v>
       </c>
       <c r="C25" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="D25">
         <v>25.400000000000002</v>
       </c>
       <c r="E25" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B26" s="22">
         <v>46063</v>
       </c>
       <c r="C26" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="D26">
         <v>11.200000000000001</v>
       </c>
       <c r="E26" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="B27" s="22">
         <v>46064</v>
       </c>
       <c r="C27" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="D27">
         <v>12.200000000000001</v>
       </c>
       <c r="E27" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="B28" s="22">
         <v>46065</v>
       </c>
       <c r="C28" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="D28">
         <v>10.600000000000001</v>
       </c>
       <c r="E28" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="B29" s="22">
         <v>46066</v>
       </c>
       <c r="C29" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="D29">
         <v>10.4</v>
       </c>
       <c r="E29" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="B30" s="22">
         <v>46067</v>
       </c>
       <c r="C30" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="D30">
         <v>25.400000000000002</v>
       </c>
       <c r="E30" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="B31" s="22">
         <v>46072</v>
       </c>
       <c r="C31" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="D31">
         <v>9.600000000000001</v>
       </c>
       <c r="E31" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="B32" s="22">
         <v>46073</v>
       </c>
       <c r="C32" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="D32">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="B33" s="22">
         <v>46074</v>
       </c>
       <c r="C33" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="D33">
         <v>26.200000000000003</v>
       </c>
       <c r="E33" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="B34" s="22">
         <v>46077</v>
       </c>
       <c r="C34" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D34">
         <v>15.8</v>
       </c>
       <c r="E34" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="B35" s="22">
         <v>46078</v>
       </c>
       <c r="C35" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="D35">
         <v>13.4</v>
       </c>
       <c r="E35" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="B36" s="22">
         <v>46079</v>
       </c>
       <c r="C36" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="D36">
         <v>11.200000000000001</v>
       </c>
       <c r="E36" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="B37" s="22">
         <v>46080</v>
       </c>
       <c r="C37" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="D37">
         <v>13.64</v>
       </c>
       <c r="E37" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="B38" s="22">
         <v>46081</v>
       </c>
       <c r="C38" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="D38">
         <v>30</v>
       </c>
       <c r="E38" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="B39" s="22">
         <v>46085</v>
       </c>
       <c r="C39" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="D39">
         <v>9.200000000000001</v>
       </c>
       <c r="E39" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="B40" s="22">
         <v>46086</v>
       </c>
       <c r="C40" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="D40">
         <v>9.600000000000001</v>
       </c>
       <c r="E40" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B41" s="22">
         <v>46087</v>
       </c>
       <c r="C41" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="D41">
         <v>8.48</v>
       </c>
       <c r="E41" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="B42" s="22">
         <v>46088</v>
       </c>
       <c r="C42" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="D42">
         <v>26.72</v>
       </c>
       <c r="E42" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="B43" s="22">
         <v>46091</v>
       </c>
       <c r="C43" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="D43">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="B44" s="22">
         <v>46092</v>
       </c>
       <c r="C44" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="D44">
         <v>11.200000000000001</v>
       </c>
       <c r="E44" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="B45" s="22">
         <v>46093</v>
       </c>
       <c r="C45" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="D45">
         <v>9</v>
       </c>
       <c r="E45" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="B46" s="22">
         <v>46094</v>
       </c>
       <c r="C46" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="D46">
         <v>10.8</v>
       </c>
       <c r="E46" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="B47" s="22">
         <v>46095</v>
       </c>
       <c r="C47" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="D47">
         <v>26.200000000000003</v>
       </c>
       <c r="E47" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="B48" s="22">
         <v>46098</v>
       </c>
       <c r="C48" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="D48">
         <v>10.8</v>
       </c>
       <c r="E48" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="B49" s="22">
         <v>46099</v>
       </c>
       <c r="C49" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="D49">
         <v>10</v>
       </c>
       <c r="E49" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="B50" s="22">
         <v>46100</v>
       </c>
       <c r="C50" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="D50">
         <v>9.600000000000001</v>
       </c>
       <c r="E50" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="B51" s="22">
         <v>46101</v>
       </c>
       <c r="C51" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="D51">
         <v>11.4</v>
       </c>
       <c r="E51" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="B52" s="22">
         <v>46102</v>
       </c>
       <c r="C52" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D52">
         <v>28.200000000000003</v>
       </c>
       <c r="E52" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="B53" s="22">
         <v>46105</v>
       </c>
       <c r="C53" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="D53">
         <v>8.6</v>
       </c>
       <c r="E53" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="B54" s="22">
         <v>46106</v>
       </c>
       <c r="C54" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="D54">
         <v>9.200000000000001</v>
       </c>
       <c r="E54" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B55" s="22">
         <v>46107</v>
       </c>
       <c r="C55" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="D55">
         <v>8.92</v>
       </c>
       <c r="E55" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="B56" s="22">
         <v>46108</v>
       </c>
       <c r="C56" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="D56">
         <v>10</v>
       </c>
       <c r="E56" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="B57" s="22">
         <v>46109</v>
       </c>
       <c r="C57" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="D57">
         <v>25.52</v>
       </c>
       <c r="E57" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="B58" s="22">
         <v>46112</v>
       </c>
       <c r="C58" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="D58">
         <v>13.200000000000001</v>
       </c>
       <c r="E58" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="B59" s="22">
         <v>46113</v>
       </c>
       <c r="C59" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="D59">
         <v>9.200000000000001</v>
       </c>
       <c r="E59" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="B60" s="22">
         <v>46114</v>
       </c>
       <c r="C60" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="D60">
         <v>9.24</v>
       </c>
       <c r="E60" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="B61" s="22">
         <v>46119</v>
       </c>
       <c r="C61" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="D61">
         <v>10.240000000000002</v>
       </c>
       <c r="E61" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="B62" s="22">
         <v>46120</v>
       </c>
       <c r="C62" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="D62">
         <v>9.28</v>
       </c>
       <c r="E62" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="B63" s="22">
         <v>46121</v>
       </c>
       <c r="C63" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="D63">
         <v>12.200000000000001</v>
       </c>
       <c r="E63" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="B64" s="22">
         <v>46122</v>
       </c>
       <c r="C64" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="D64">
         <v>9.24</v>
       </c>
       <c r="E64" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="B65" s="22">
         <v>46123</v>
       </c>
       <c r="C65" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="D65">
         <v>25.400000000000002</v>
       </c>
       <c r="E65" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="B66" s="22">
         <v>46126</v>
       </c>
       <c r="C66" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="D66">
         <v>14</v>
       </c>
       <c r="E66" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="B67" s="22">
         <v>46127</v>
       </c>
       <c r="C67" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="D67">
         <v>8.6</v>
       </c>
       <c r="E67" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="B68" s="22">
         <v>46128</v>
       </c>
       <c r="C68" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="D68">
         <v>8.8</v>
       </c>
       <c r="E68" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="B69" s="22">
         <v>46129</v>
       </c>
       <c r="C69" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="D69">
         <v>8.8</v>
       </c>
       <c r="E69" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="B70" s="22">
         <v>46130</v>
       </c>
       <c r="C70" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D70">
         <v>25.200000000000003</v>
       </c>
       <c r="E70" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="B71" s="22">
         <v>46134</v>
       </c>
       <c r="C71" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="D71">
         <v>10.4</v>
       </c>
       <c r="E71" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="B72" s="22">
         <v>46135</v>
       </c>
       <c r="C72" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="D72">
         <v>8.88</v>
       </c>
       <c r="E72" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="B73" s="22">
         <v>46136</v>
       </c>
       <c r="C73" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="D73">
         <v>11</v>
       </c>
       <c r="E73" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B74" s="22">
         <v>46137</v>
       </c>
       <c r="C74" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="D74">
         <v>25.200000000000003</v>
       </c>
       <c r="E74" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="B75" s="22">
         <v>46140</v>
       </c>
       <c r="C75" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="D75">
         <v>12.960000000000003</v>
       </c>
       <c r="E75" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="B76" s="22">
         <v>46141</v>
       </c>
       <c r="C76" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="D76">
         <v>9.8</v>
       </c>
       <c r="E76" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="B77" s="22">
         <v>46142</v>
       </c>
       <c r="C77" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="D77">
         <v>10.280000000000001</v>
       </c>
       <c r="E77" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="B78" s="22">
         <v>46144</v>
       </c>
       <c r="C78" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="D78">
         <v>19.28</v>
       </c>
       <c r="E78" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="B79" s="22">
         <v>46147</v>
       </c>
       <c r="C79" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="D79">
         <v>7.800000000000001</v>
       </c>
       <c r="E79" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="B80" s="22">
         <v>46148</v>
       </c>
       <c r="C80" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="D80">
         <v>7.4</v>
       </c>
       <c r="E80" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="B81" s="22">
         <v>46149</v>
       </c>
       <c r="C81" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="D81">
         <v>7.800000000000001</v>
       </c>
       <c r="E81" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="B82" s="22">
         <v>46154</v>
       </c>
       <c r="C82" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="D82">
         <v>13.4</v>
       </c>
       <c r="E82" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="B83" s="22">
         <v>46155</v>
       </c>
       <c r="C83" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="D83">
         <v>9</v>
       </c>
       <c r="E83" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="B84" s="22">
         <v>46156</v>
       </c>
       <c r="C84" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D84">
         <v>8.4</v>
       </c>
       <c r="E84" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="B85" s="22">
         <v>46157</v>
       </c>
       <c r="C85" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="D85">
         <v>9.200000000000001</v>
       </c>
       <c r="E85" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="B86" s="22">
         <v>46158</v>
       </c>
       <c r="C86" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="D86">
         <v>18</v>
       </c>
       <c r="E86" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="B87" s="22">
         <v>46161</v>
       </c>
       <c r="C87" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="D87">
         <v>8</v>
       </c>
       <c r="E87" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="B88" s="22">
         <v>46162</v>
       </c>
       <c r="C88" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="D88">
         <v>11.8</v>
       </c>
       <c r="E88" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="B89" s="22">
         <v>46163</v>
       </c>
       <c r="C89" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="D89">
         <v>9.200000000000001</v>
       </c>
       <c r="E89" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="B90" s="22">
         <v>46164</v>
       </c>
       <c r="C90" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="D90">
         <v>10.8</v>
       </c>
       <c r="E90" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="B91" s="22">
         <v>46165</v>
       </c>
       <c r="C91" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="D91">
         <v>26.080000000000002</v>
       </c>
       <c r="E91" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -11054,16 +11116,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="G3" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -11077,7 +11139,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F4" s="8">
         <v>1333</v>
@@ -11097,7 +11159,7 @@
         <v>58.999999999999986</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="F5" s="8">
         <v>1271.2</v>
@@ -11117,7 +11179,7 @@
         <v>46</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="F6" s="8">
         <v>1343.1999999999998</v>
@@ -11137,7 +11199,7 @@
         <v>44</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="F7" s="8">
         <v>1193.6000000000001</v>
@@ -11157,7 +11219,7 @@
         <v>47.999999999999986</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="F8" s="8">
         <v>1155.2</v>
@@ -11177,7 +11239,7 @@
         <v>127.4</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="F9" s="8">
         <v>0</v>
@@ -11197,7 +11259,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="F10" s="8">
         <v>0</v>
@@ -11208,14 +11270,14 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="20">
         <v>324.4</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -11226,7 +11288,7 @@
     </row>
     <row r="12" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E12" s="1" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -11237,7 +11299,7 @@
     </row>
     <row r="13" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E13" s="1" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F13" s="8">
         <v>0</v>
@@ -11248,7 +11310,7 @@
     </row>
     <row r="14" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E14" s="1" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="F14" s="8">
         <v>0</v>
@@ -11259,7 +11321,7 @@
     </row>
     <row r="15" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E15" s="1" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="F15" s="8">
         <v>0</v>
@@ -11270,7 +11332,7 @@
     </row>
     <row r="16" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E16" s="1" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="F16" s="8">
         <v>6296.2</v>

</xml_diff>

<commit_message>
fix(cache): solve local PWA caching issues and fix yesterday's shift data
</commit_message>
<xml_diff>
--- a/Controle_de_Horas_Trabalho-1.xlsx
+++ b/Controle_de_Horas_Trabalho-1.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="270">
   <si>
     <t>Data</t>
   </si>
@@ -166,13 +166,7 @@
     <t>12:15</t>
   </si>
   <si>
-    <t>13:15</t>
-  </si>
-  <si>
-    <t>17:15</t>
-  </si>
-  <si>
-    <t>Teste API</t>
+    <t>Cleared second shift test</t>
   </si>
   <si>
     <t>Pendente</t>
@@ -181,13 +175,13 @@
     <t>07:15</t>
   </si>
   <si>
-    <t>17:45</t>
+    <t>12:45</t>
   </si>
   <si>
     <t>01:30</t>
   </si>
   <si>
-    <t>10:30</t>
+    <t>05:30</t>
   </si>
   <si>
     <t>Soma de Valor do Dia (R$)</t>
@@ -797,6 +791,42 @@
   </si>
   <si>
     <t>Ponto de 2026-05-23</t>
+  </si>
+  <si>
+    <t>auto_inv_178061283292416</t>
+  </si>
+  <si>
+    <t>Ponto de 2026-05-26</t>
+  </si>
+  <si>
+    <t>auto_inv_17806128329257</t>
+  </si>
+  <si>
+    <t>Ponto de 2026-05-27</t>
+  </si>
+  <si>
+    <t>auto_inv_178061283292514</t>
+  </si>
+  <si>
+    <t>Ponto de 2026-05-28</t>
+  </si>
+  <si>
+    <t>auto_inv_178061283292524</t>
+  </si>
+  <si>
+    <t>Ponto de 2026-05-29</t>
+  </si>
+  <si>
+    <t>auto_inv_178061283292531</t>
+  </si>
+  <si>
+    <t>Ponto de 2026-05-30</t>
+  </si>
+  <si>
+    <t>auto_inv_178061283292525</t>
+  </si>
+  <si>
+    <t>Ponto de 2026-05-31</t>
   </si>
 </sst>
 </file>
@@ -5029,13 +5059,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="145" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="145" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A145" s="6">
         <v>46166</v>
       </c>
       <c r="B145" t="s">
         <v>19</v>
       </c>
+      <c r="C145" s="1"/>
+      <c r="D145" s="1"/>
+      <c r="E145" s="1"/>
+      <c r="F145" s="1"/>
       <c r="G145" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -5044,14 +5078,21 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="146" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K145" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="146" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A146" s="6">
         <v>46167</v>
       </c>
       <c r="B146" t="s">
         <v>20</v>
       </c>
+      <c r="C146" s="1"/>
+      <c r="D146" s="1"/>
+      <c r="E146" s="1"/>
+      <c r="F146" s="1"/>
       <c r="G146" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -5060,8 +5101,11 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="147" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K146" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="147" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A147" s="6">
         <v>46168</v>
       </c>
@@ -5074,6 +5118,8 @@
       <c r="D147" s="9">
         <v>0.9166666666678793</v>
       </c>
+      <c r="E147" s="1"/>
+      <c r="F147" s="1"/>
       <c r="G147" s="7">
         <f t="shared" si="4"/>
         <v>0.20486111110949423</v>
@@ -5082,8 +5128,11 @@
         <f t="shared" si="5"/>
         <v>58.999999999999986</v>
       </c>
-    </row>
-    <row r="148" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K147" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="148" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A148" s="6">
         <v>46169</v>
       </c>
@@ -5096,6 +5145,8 @@
       <c r="D148" s="9">
         <v>0.875</v>
       </c>
+      <c r="E148" s="1"/>
+      <c r="F148" s="1"/>
       <c r="G148" s="7">
         <f t="shared" si="4"/>
         <v>0.15972222222262644</v>
@@ -5104,8 +5155,11 @@
         <f t="shared" si="5"/>
         <v>46</v>
       </c>
-    </row>
-    <row r="149" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K148" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="149" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A149" s="6">
         <v>46170</v>
       </c>
@@ -5118,6 +5172,8 @@
       <c r="D149" s="9">
         <v>0.875</v>
       </c>
+      <c r="E149" s="1"/>
+      <c r="F149" s="1"/>
       <c r="G149" s="7">
         <f t="shared" si="4"/>
         <v>0.15277777777737356</v>
@@ -5126,8 +5182,11 @@
         <f t="shared" si="5"/>
         <v>44</v>
       </c>
-    </row>
-    <row r="150" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K149" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="150" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A150" s="6">
         <v>46171</v>
       </c>
@@ -5140,6 +5199,8 @@
       <c r="D150" s="9">
         <v>0.8819444444452529</v>
       </c>
+      <c r="E150" s="1"/>
+      <c r="F150" s="1"/>
       <c r="G150" s="7">
         <f t="shared" si="4"/>
         <v>0.16666666666787933</v>
@@ -5148,8 +5209,11 @@
         <f t="shared" si="5"/>
         <v>47.999999999999986</v>
       </c>
-    </row>
-    <row r="151" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K150" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="151" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A151" s="6">
         <v>46172</v>
       </c>
@@ -5176,8 +5240,11 @@
         <f t="shared" si="5"/>
         <v>127.4</v>
       </c>
-    </row>
-    <row r="152" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K151" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="152" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A152" s="6">
         <v>46173</v>
       </c>
@@ -5200,6 +5267,9 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
+      <c r="K152" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="153" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" s="6">
@@ -5246,39 +5316,35 @@
       <c r="D155" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E155" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F155" s="1" t="s">
-        <v>50</v>
-      </c>
+      <c r="E155" s="1"/>
+      <c r="F155" s="1"/>
       <c r="G155" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H155" s="8">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="I155">
         <v>12</v>
       </c>
       <c r="J155" t="s">
+        <v>49</v>
+      </c>
+      <c r="K155" t="s">
+        <v>50</v>
+      </c>
+      <c r="L155" t="s">
         <v>51</v>
       </c>
-      <c r="K155" t="s">
+      <c r="M155" t="s">
         <v>52</v>
       </c>
-      <c r="L155" t="s">
+      <c r="N155" t="s">
         <v>53</v>
       </c>
-      <c r="M155" t="s">
+      <c r="O155" t="s">
         <v>54</v>
-      </c>
-      <c r="N155" t="s">
-        <v>55</v>
-      </c>
-      <c r="O155" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="156" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9374,22 +9440,22 @@
   <sheetData>
     <row r="1" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="21" t="s">
+      <c r="E1" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="F1" s="21" t="s">
         <v>75</v>
-      </c>
-      <c r="E1" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="F1" s="21" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -9400,1554 +9466,1656 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="21" t="s">
         <v>73</v>
-      </c>
-      <c r="B1" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="D1" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="E1" s="21" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B2" s="22">
         <v>46028</v>
       </c>
       <c r="C2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D2">
         <v>9.8</v>
       </c>
       <c r="E2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B3" s="22">
         <v>46029</v>
       </c>
       <c r="C3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D3">
         <v>12.4</v>
       </c>
       <c r="E3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B4" s="22">
         <v>46030</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D4">
         <v>10.4</v>
       </c>
       <c r="E4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B5" s="22">
         <v>46031</v>
       </c>
       <c r="C5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D5">
         <v>9.4</v>
       </c>
       <c r="E5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B6" s="22">
         <v>46032</v>
       </c>
       <c r="C6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D6">
-        <v>26.200000000000003</v>
+        <v>26.2</v>
       </c>
       <c r="E6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B7" s="22">
         <v>46035</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D7">
         <v>9.4</v>
       </c>
       <c r="E7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B8" s="22">
         <v>46036</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D8">
-        <v>9.600000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="E8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B9" s="22">
         <v>46037</v>
       </c>
       <c r="C9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D9">
         <v>11.8</v>
       </c>
       <c r="E9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B10" s="22">
         <v>46038</v>
       </c>
       <c r="C10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D10">
-        <v>10.200000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="E10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B11" s="22">
         <v>46039</v>
       </c>
       <c r="C11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D11">
         <v>24.32</v>
       </c>
       <c r="E11" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B12" s="22">
         <v>46042</v>
       </c>
       <c r="C12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D12">
         <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B13" s="22">
         <v>46043</v>
       </c>
       <c r="C13" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D13">
         <v>11.8</v>
       </c>
       <c r="E13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B14" s="22">
         <v>46044</v>
       </c>
       <c r="C14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D14">
         <v>9.4</v>
       </c>
       <c r="E14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B15" s="22">
         <v>46045</v>
       </c>
       <c r="C15" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D15">
-        <v>10.200000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="E15" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B16" s="22">
         <v>46046</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D16">
         <v>18.6</v>
       </c>
       <c r="E16" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B17" s="22">
         <v>46049</v>
       </c>
       <c r="C17" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D17">
         <v>16.6</v>
       </c>
       <c r="E17" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B18" s="22">
         <v>46050</v>
       </c>
       <c r="C18" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D18">
-        <v>11.200000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="E18" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B19" s="22">
         <v>46051</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D19">
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B20" s="22">
         <v>46052</v>
       </c>
       <c r="C20" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D20">
-        <v>11.280000000000001</v>
+        <v>11.28</v>
       </c>
       <c r="E20" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B21" s="22">
         <v>46053</v>
       </c>
       <c r="C21" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D21">
         <v>24</v>
       </c>
       <c r="E21" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B22" s="22">
         <v>46057</v>
       </c>
       <c r="C22" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D22">
         <v>8.6</v>
       </c>
       <c r="E22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B23" s="22">
         <v>46058</v>
       </c>
       <c r="C23" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D23">
         <v>9.4</v>
       </c>
       <c r="E23" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B24" s="22">
         <v>46059</v>
       </c>
       <c r="C24" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D24">
-        <v>10.200000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="E24" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B25" s="22">
         <v>46060</v>
       </c>
       <c r="C25" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D25">
-        <v>25.400000000000002</v>
+        <v>25.4</v>
       </c>
       <c r="E25" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B26" s="22">
         <v>46063</v>
       </c>
       <c r="C26" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D26">
-        <v>11.200000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="E26" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B27" s="22">
         <v>46064</v>
       </c>
       <c r="C27" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D27">
-        <v>12.200000000000001</v>
+        <v>12.2</v>
       </c>
       <c r="E27" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B28" s="22">
         <v>46065</v>
       </c>
       <c r="C28" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D28">
-        <v>10.600000000000001</v>
+        <v>10.6</v>
       </c>
       <c r="E28" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B29" s="22">
         <v>46066</v>
       </c>
       <c r="C29" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D29">
         <v>10.4</v>
       </c>
       <c r="E29" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B30" s="22">
         <v>46067</v>
       </c>
       <c r="C30" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D30">
-        <v>25.400000000000002</v>
+        <v>25.4</v>
       </c>
       <c r="E30" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B31" s="22">
         <v>46072</v>
       </c>
       <c r="C31" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D31">
-        <v>9.600000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="E31" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B32" s="22">
         <v>46073</v>
       </c>
       <c r="C32" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D32">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B33" s="22">
         <v>46074</v>
       </c>
       <c r="C33" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D33">
-        <v>26.200000000000003</v>
+        <v>26.2</v>
       </c>
       <c r="E33" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B34" s="22">
         <v>46077</v>
       </c>
       <c r="C34" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D34">
         <v>15.8</v>
       </c>
       <c r="E34" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B35" s="22">
         <v>46078</v>
       </c>
       <c r="C35" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D35">
         <v>13.4</v>
       </c>
       <c r="E35" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B36" s="22">
         <v>46079</v>
       </c>
       <c r="C36" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D36">
-        <v>11.200000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="E36" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B37" s="22">
         <v>46080</v>
       </c>
       <c r="C37" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D37">
         <v>13.64</v>
       </c>
       <c r="E37" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B38" s="22">
         <v>46081</v>
       </c>
       <c r="C38" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D38">
         <v>30</v>
       </c>
       <c r="E38" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B39" s="22">
         <v>46085</v>
       </c>
       <c r="C39" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D39">
-        <v>9.200000000000001</v>
+        <v>9.2</v>
       </c>
       <c r="E39" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B40" s="22">
         <v>46086</v>
       </c>
       <c r="C40" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D40">
-        <v>9.600000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="E40" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B41" s="22">
         <v>46087</v>
       </c>
       <c r="C41" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D41">
         <v>8.48</v>
       </c>
       <c r="E41" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B42" s="22">
         <v>46088</v>
       </c>
       <c r="C42" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D42">
         <v>26.72</v>
       </c>
       <c r="E42" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B43" s="22">
         <v>46091</v>
       </c>
       <c r="C43" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D43">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B44" s="22">
         <v>46092</v>
       </c>
       <c r="C44" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D44">
-        <v>11.200000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="E44" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B45" s="22">
         <v>46093</v>
       </c>
       <c r="C45" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D45">
         <v>9</v>
       </c>
       <c r="E45" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B46" s="22">
         <v>46094</v>
       </c>
       <c r="C46" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D46">
         <v>10.8</v>
       </c>
       <c r="E46" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B47" s="22">
         <v>46095</v>
       </c>
       <c r="C47" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D47">
-        <v>26.200000000000003</v>
+        <v>26.2</v>
       </c>
       <c r="E47" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B48" s="22">
         <v>46098</v>
       </c>
       <c r="C48" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D48">
         <v>10.8</v>
       </c>
       <c r="E48" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B49" s="22">
         <v>46099</v>
       </c>
       <c r="C49" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D49">
         <v>10</v>
       </c>
       <c r="E49" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B50" s="22">
         <v>46100</v>
       </c>
       <c r="C50" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D50">
-        <v>9.600000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="E50" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B51" s="22">
         <v>46101</v>
       </c>
       <c r="C51" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D51">
         <v>11.4</v>
       </c>
       <c r="E51" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B52" s="22">
         <v>46102</v>
       </c>
       <c r="C52" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D52">
-        <v>28.200000000000003</v>
+        <v>28.2</v>
       </c>
       <c r="E52" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B53" s="22">
         <v>46105</v>
       </c>
       <c r="C53" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D53">
         <v>8.6</v>
       </c>
       <c r="E53" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B54" s="22">
         <v>46106</v>
       </c>
       <c r="C54" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D54">
-        <v>9.200000000000001</v>
+        <v>9.2</v>
       </c>
       <c r="E54" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B55" s="22">
         <v>46107</v>
       </c>
       <c r="C55" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D55">
         <v>8.92</v>
       </c>
       <c r="E55" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B56" s="22">
         <v>46108</v>
       </c>
       <c r="C56" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D56">
         <v>10</v>
       </c>
       <c r="E56" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B57" s="22">
         <v>46109</v>
       </c>
       <c r="C57" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D57">
         <v>25.52</v>
       </c>
       <c r="E57" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B58" s="22">
         <v>46112</v>
       </c>
       <c r="C58" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D58">
-        <v>13.200000000000001</v>
+        <v>13.2</v>
       </c>
       <c r="E58" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B59" s="22">
         <v>46113</v>
       </c>
       <c r="C59" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D59">
-        <v>9.200000000000001</v>
+        <v>9.2</v>
       </c>
       <c r="E59" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B60" s="22">
         <v>46114</v>
       </c>
       <c r="C60" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D60">
         <v>9.24</v>
       </c>
       <c r="E60" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B61" s="22">
         <v>46119</v>
       </c>
       <c r="C61" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D61">
-        <v>10.240000000000002</v>
+        <v>10.24</v>
       </c>
       <c r="E61" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B62" s="22">
         <v>46120</v>
       </c>
       <c r="C62" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D62">
         <v>9.28</v>
       </c>
       <c r="E62" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B63" s="22">
         <v>46121</v>
       </c>
       <c r="C63" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D63">
-        <v>12.200000000000001</v>
+        <v>12.2</v>
       </c>
       <c r="E63" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B64" s="22">
         <v>46122</v>
       </c>
       <c r="C64" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D64">
         <v>9.24</v>
       </c>
       <c r="E64" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B65" s="22">
         <v>46123</v>
       </c>
       <c r="C65" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D65">
-        <v>25.400000000000002</v>
+        <v>25.4</v>
       </c>
       <c r="E65" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B66" s="22">
         <v>46126</v>
       </c>
       <c r="C66" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D66">
         <v>14</v>
       </c>
       <c r="E66" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B67" s="22">
         <v>46127</v>
       </c>
       <c r="C67" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D67">
         <v>8.6</v>
       </c>
       <c r="E67" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B68" s="22">
         <v>46128</v>
       </c>
       <c r="C68" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D68">
         <v>8.8</v>
       </c>
       <c r="E68" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B69" s="22">
         <v>46129</v>
       </c>
       <c r="C69" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D69">
         <v>8.8</v>
       </c>
       <c r="E69" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B70" s="22">
         <v>46130</v>
       </c>
       <c r="C70" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D70">
-        <v>25.200000000000003</v>
+        <v>25.2</v>
       </c>
       <c r="E70" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B71" s="22">
         <v>46134</v>
       </c>
       <c r="C71" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D71">
         <v>10.4</v>
       </c>
       <c r="E71" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B72" s="22">
         <v>46135</v>
       </c>
       <c r="C72" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D72">
         <v>8.88</v>
       </c>
       <c r="E72" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B73" s="22">
         <v>46136</v>
       </c>
       <c r="C73" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D73">
         <v>11</v>
       </c>
       <c r="E73" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B74" s="22">
         <v>46137</v>
       </c>
       <c r="C74" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D74">
-        <v>25.200000000000003</v>
+        <v>25.2</v>
       </c>
       <c r="E74" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B75" s="22">
         <v>46140</v>
       </c>
       <c r="C75" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D75">
-        <v>12.960000000000003</v>
+        <v>12.96</v>
       </c>
       <c r="E75" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B76" s="22">
         <v>46141</v>
       </c>
       <c r="C76" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D76">
         <v>9.8</v>
       </c>
       <c r="E76" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B77" s="22">
         <v>46142</v>
       </c>
       <c r="C77" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D77">
-        <v>10.280000000000001</v>
+        <v>10.28</v>
       </c>
       <c r="E77" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B78" s="22">
         <v>46144</v>
       </c>
       <c r="C78" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D78">
         <v>19.28</v>
       </c>
       <c r="E78" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B79" s="22">
         <v>46147</v>
       </c>
       <c r="C79" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D79">
-        <v>7.800000000000001</v>
+        <v>7.8</v>
       </c>
       <c r="E79" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B80" s="22">
         <v>46148</v>
       </c>
       <c r="C80" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D80">
         <v>7.4</v>
       </c>
       <c r="E80" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B81" s="22">
         <v>46149</v>
       </c>
       <c r="C81" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D81">
-        <v>7.800000000000001</v>
+        <v>7.8</v>
       </c>
       <c r="E81" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B82" s="22">
         <v>46154</v>
       </c>
       <c r="C82" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D82">
         <v>13.4</v>
       </c>
       <c r="E82" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B83" s="22">
         <v>46155</v>
       </c>
       <c r="C83" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D83">
         <v>9</v>
       </c>
       <c r="E83" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B84" s="22">
         <v>46156</v>
       </c>
       <c r="C84" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D84">
         <v>8.4</v>
       </c>
       <c r="E84" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B85" s="22">
         <v>46157</v>
       </c>
       <c r="C85" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D85">
-        <v>9.200000000000001</v>
+        <v>9.2</v>
       </c>
       <c r="E85" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B86" s="22">
         <v>46158</v>
       </c>
       <c r="C86" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D86">
         <v>18</v>
       </c>
       <c r="E86" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B87" s="22">
         <v>46161</v>
       </c>
       <c r="C87" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D87">
         <v>8</v>
       </c>
       <c r="E87" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B88" s="22">
         <v>46162</v>
       </c>
       <c r="C88" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D88">
         <v>11.8</v>
       </c>
       <c r="E88" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B89" s="22">
         <v>46163</v>
       </c>
       <c r="C89" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D89">
-        <v>9.200000000000001</v>
+        <v>9.2</v>
       </c>
       <c r="E89" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B90" s="22">
         <v>46164</v>
       </c>
       <c r="C90" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D90">
         <v>10.8</v>
       </c>
       <c r="E90" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B91" s="22">
         <v>46165</v>
       </c>
       <c r="C91" t="s">
+        <v>257</v>
+      </c>
+      <c r="D91">
+        <v>26.08</v>
+      </c>
+      <c r="E91" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>258</v>
+      </c>
+      <c r="B92" s="22">
+        <v>46168</v>
+      </c>
+      <c r="C92" t="s">
         <v>259</v>
       </c>
-      <c r="D91">
-        <v>26.080000000000002</v>
-      </c>
-      <c r="E91" t="s">
-        <v>81</v>
+      <c r="D92">
+        <v>11.8</v>
+      </c>
+      <c r="E92" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>260</v>
+      </c>
+      <c r="B93" s="22">
+        <v>46169</v>
+      </c>
+      <c r="C93" t="s">
+        <v>261</v>
+      </c>
+      <c r="D93">
+        <v>9.2</v>
+      </c>
+      <c r="E93" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>262</v>
+      </c>
+      <c r="B94" s="22">
+        <v>46170</v>
+      </c>
+      <c r="C94" t="s">
+        <v>263</v>
+      </c>
+      <c r="D94">
+        <v>8.8</v>
+      </c>
+      <c r="E94" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>264</v>
+      </c>
+      <c r="B95" s="22">
+        <v>46171</v>
+      </c>
+      <c r="C95" t="s">
+        <v>265</v>
+      </c>
+      <c r="D95">
+        <v>9.6</v>
+      </c>
+      <c r="E95" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>266</v>
+      </c>
+      <c r="B96" s="22">
+        <v>46172</v>
+      </c>
+      <c r="C96" t="s">
+        <v>267</v>
+      </c>
+      <c r="D96">
+        <v>25.48</v>
+      </c>
+      <c r="E96" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>268</v>
+      </c>
+      <c r="B97" s="22">
+        <v>46173</v>
+      </c>
+      <c r="C97" t="s">
+        <v>269</v>
+      </c>
+      <c r="D97">
+        <v>0.04</v>
+      </c>
+      <c r="E97" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -11116,16 +11284,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" t="s">
         <v>57</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="F3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -11139,7 +11307,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F4" s="8">
         <v>1333</v>
@@ -11159,7 +11327,7 @@
         <v>58.999999999999986</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F5" s="8">
         <v>1271.2</v>
@@ -11179,7 +11347,7 @@
         <v>46</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F6" s="8">
         <v>1343.1999999999998</v>
@@ -11199,7 +11367,7 @@
         <v>44</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F7" s="8">
         <v>1193.6000000000001</v>
@@ -11219,7 +11387,7 @@
         <v>47.999999999999986</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F8" s="8">
         <v>1155.2</v>
@@ -11239,7 +11407,7 @@
         <v>127.4</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F9" s="8">
         <v>0</v>
@@ -11259,7 +11427,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F10" s="8">
         <v>0</v>
@@ -11270,14 +11438,14 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="20">
         <v>324.4</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -11288,7 +11456,7 @@
     </row>
     <row r="12" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E12" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -11299,7 +11467,7 @@
     </row>
     <row r="13" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E13" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F13" s="8">
         <v>0</v>
@@ -11310,7 +11478,7 @@
     </row>
     <row r="14" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E14" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F14" s="8">
         <v>0</v>
@@ -11321,7 +11489,7 @@
     </row>
     <row r="15" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E15" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F15" s="8">
         <v>0</v>
@@ -11332,7 +11500,7 @@
     </row>
     <row r="16" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E16" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F16" s="8">
         <v>6296.2</v>

</xml_diff>

<commit_message>
fix: implement server-side mobile redirect to permanent origin for persistent localStorage
</commit_message>
<xml_diff>
--- a/Controle_de_Horas_Trabalho-1.xlsx
+++ b/Controle_de_Horas_Trabalho-1.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="274">
   <si>
     <t>Data</t>
   </si>
@@ -160,28 +160,40 @@
     <t>08:24</t>
   </si>
   <si>
-    <t>08:15</t>
-  </si>
-  <si>
-    <t>12:15</t>
+    <t>17:15</t>
+  </si>
+  <si>
+    <t>Pendente</t>
+  </si>
+  <si>
+    <t>17:03</t>
   </si>
   <si>
     <t>Cleared second shift test</t>
   </si>
   <si>
-    <t>Pendente</t>
-  </si>
-  <si>
-    <t>07:15</t>
-  </si>
-  <si>
-    <t>12:45</t>
-  </si>
-  <si>
-    <t>01:30</t>
-  </si>
-  <si>
-    <t>05:30</t>
+    <t>17:17</t>
+  </si>
+  <si>
+    <t>08:55</t>
+  </si>
+  <si>
+    <t>13:44</t>
+  </si>
+  <si>
+    <t>21:55</t>
+  </si>
+  <si>
+    <t>17:33</t>
+  </si>
+  <si>
+    <t>17:39</t>
+  </si>
+  <si>
+    <t>22:10</t>
+  </si>
+  <si>
+    <t>08:30</t>
   </si>
   <si>
     <t>Soma de Valor do Dia (R$)</t>
@@ -5287,23 +5299,33 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="154" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A154" s="6">
         <v>46175</v>
       </c>
       <c r="B154" t="s">
         <v>21</v>
       </c>
+      <c r="C154" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D154" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E154" s="1"/>
+      <c r="F154" s="1"/>
       <c r="G154" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H154" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="155" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="K154" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="155" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A155" s="6">
         <v>46176</v>
       </c>
@@ -5311,10 +5333,10 @@
         <v>24</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="E155" s="1"/>
       <c r="F155" s="1"/>
@@ -5323,28 +5345,16 @@
         <v>0</v>
       </c>
       <c r="H155" s="8">
-        <v>48</v>
+        <v>47.4</v>
       </c>
       <c r="I155">
         <v>12</v>
       </c>
       <c r="J155" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K155" t="s">
-        <v>50</v>
-      </c>
-      <c r="L155" t="s">
-        <v>51</v>
-      </c>
-      <c r="M155" t="s">
-        <v>52</v>
-      </c>
-      <c r="N155" t="s">
-        <v>53</v>
-      </c>
-      <c r="O155" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="156" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5363,36 +5373,60 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="157" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A157" s="6">
         <v>46178</v>
       </c>
       <c r="B157" t="s">
         <v>17</v>
       </c>
+      <c r="C157" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D157" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E157" s="1"/>
+      <c r="F157" s="1"/>
       <c r="G157" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H157" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+        <v>44.6</v>
+      </c>
+      <c r="K157" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="158" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A158" s="6">
         <v>46179</v>
       </c>
       <c r="B158" t="s">
         <v>18</v>
       </c>
+      <c r="C158" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D158" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E158" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F158" s="1" t="s">
+        <v>28</v>
+      </c>
       <c r="G158" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H158" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>124.2</v>
+      </c>
+      <c r="K158" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="159" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5427,84 +5461,138 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="161" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161" s="6">
         <v>46182</v>
       </c>
       <c r="B161" t="s">
         <v>21</v>
       </c>
+      <c r="C161" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D161" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E161" s="1"/>
+      <c r="F161" s="1"/>
       <c r="G161" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H161" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="162" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+        <v>55.6</v>
+      </c>
+      <c r="K161" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="162" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" s="6">
         <v>46183</v>
       </c>
       <c r="B162" t="s">
         <v>24</v>
       </c>
+      <c r="C162" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D162" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E162" s="1"/>
+      <c r="F162" s="1"/>
       <c r="G162" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H162" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="163" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+        <v>41.4</v>
+      </c>
+      <c r="K162" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="163" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163" s="6">
         <v>46184</v>
       </c>
       <c r="B163" t="s">
         <v>15</v>
       </c>
+      <c r="C163" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D163" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E163" s="1"/>
+      <c r="F163" s="1"/>
       <c r="G163" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H163" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="164" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+        <v>40.2</v>
+      </c>
+      <c r="K163" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="164" ht="15.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164" s="6">
         <v>46185</v>
       </c>
       <c r="B164" t="s">
         <v>17</v>
       </c>
+      <c r="C164" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D164" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E164" s="1"/>
+      <c r="F164" s="1"/>
       <c r="G164" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H164" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="165" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+        <v>58.6</v>
+      </c>
+      <c r="K164" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="165" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A165" s="6">
         <v>46186</v>
       </c>
       <c r="B165" t="s">
         <v>18</v>
       </c>
+      <c r="C165" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D165" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E165" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F165" s="1" t="s">
+        <v>28</v>
+      </c>
       <c r="G165" s="7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H165" s="8">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>132</v>
+      </c>
+      <c r="K165" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="166" ht="15.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9440,22 +9528,22 @@
   <sheetData>
     <row r="1" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -9471,1651 +9559,1651 @@
   <sheetData>
     <row r="1" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B2" s="22">
         <v>46028</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D2">
         <v>9.8</v>
       </c>
       <c r="E2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B3" s="22">
         <v>46029</v>
       </c>
       <c r="C3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D3">
         <v>12.4</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B4" s="22">
         <v>46030</v>
       </c>
       <c r="C4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D4">
         <v>10.4</v>
       </c>
       <c r="E4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B5" s="22">
         <v>46031</v>
       </c>
       <c r="C5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D5">
         <v>9.4</v>
       </c>
       <c r="E5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B6" s="22">
         <v>46032</v>
       </c>
       <c r="C6" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D6">
         <v>26.2</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B7" s="22">
         <v>46035</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D7">
         <v>9.4</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B8" s="22">
         <v>46036</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D8">
         <v>9.6</v>
       </c>
       <c r="E8" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B9" s="22">
         <v>46037</v>
       </c>
       <c r="C9" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D9">
         <v>11.8</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B10" s="22">
         <v>46038</v>
       </c>
       <c r="C10" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D10">
         <v>10.2</v>
       </c>
       <c r="E10" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B11" s="22">
         <v>46039</v>
       </c>
       <c r="C11" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D11">
         <v>24.32</v>
       </c>
       <c r="E11" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B12" s="22">
         <v>46042</v>
       </c>
       <c r="C12" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D12">
         <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B13" s="22">
         <v>46043</v>
       </c>
       <c r="C13" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D13">
         <v>11.8</v>
       </c>
       <c r="E13" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B14" s="22">
         <v>46044</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D14">
         <v>9.4</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B15" s="22">
         <v>46045</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D15">
         <v>10.2</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B16" s="22">
         <v>46046</v>
       </c>
       <c r="C16" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D16">
         <v>18.6</v>
       </c>
       <c r="E16" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B17" s="22">
         <v>46049</v>
       </c>
       <c r="C17" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D17">
         <v>16.6</v>
       </c>
       <c r="E17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B18" s="22">
         <v>46050</v>
       </c>
       <c r="C18" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D18">
         <v>11.2</v>
       </c>
       <c r="E18" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B19" s="22">
         <v>46051</v>
       </c>
       <c r="C19" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D19">
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B20" s="22">
         <v>46052</v>
       </c>
       <c r="C20" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D20">
         <v>11.28</v>
       </c>
       <c r="E20" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B21" s="22">
         <v>46053</v>
       </c>
       <c r="C21" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D21">
         <v>24</v>
       </c>
       <c r="E21" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B22" s="22">
         <v>46057</v>
       </c>
       <c r="C22" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D22">
         <v>8.6</v>
       </c>
       <c r="E22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B23" s="22">
         <v>46058</v>
       </c>
       <c r="C23" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D23">
         <v>9.4</v>
       </c>
       <c r="E23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B24" s="22">
         <v>46059</v>
       </c>
       <c r="C24" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D24">
         <v>10.2</v>
       </c>
       <c r="E24" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B25" s="22">
         <v>46060</v>
       </c>
       <c r="C25" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D25">
         <v>25.4</v>
       </c>
       <c r="E25" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B26" s="22">
         <v>46063</v>
       </c>
       <c r="C26" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D26">
         <v>11.2</v>
       </c>
       <c r="E26" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B27" s="22">
         <v>46064</v>
       </c>
       <c r="C27" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D27">
         <v>12.2</v>
       </c>
       <c r="E27" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B28" s="22">
         <v>46065</v>
       </c>
       <c r="C28" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D28">
         <v>10.6</v>
       </c>
       <c r="E28" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B29" s="22">
         <v>46066</v>
       </c>
       <c r="C29" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D29">
         <v>10.4</v>
       </c>
       <c r="E29" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B30" s="22">
         <v>46067</v>
       </c>
       <c r="C30" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D30">
         <v>25.4</v>
       </c>
       <c r="E30" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B31" s="22">
         <v>46072</v>
       </c>
       <c r="C31" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D31">
         <v>9.6</v>
       </c>
       <c r="E31" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B32" s="22">
         <v>46073</v>
       </c>
       <c r="C32" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D32">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B33" s="22">
         <v>46074</v>
       </c>
       <c r="C33" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D33">
         <v>26.2</v>
       </c>
       <c r="E33" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B34" s="22">
         <v>46077</v>
       </c>
       <c r="C34" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D34">
         <v>15.8</v>
       </c>
       <c r="E34" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B35" s="22">
         <v>46078</v>
       </c>
       <c r="C35" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D35">
         <v>13.4</v>
       </c>
       <c r="E35" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B36" s="22">
         <v>46079</v>
       </c>
       <c r="C36" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D36">
         <v>11.2</v>
       </c>
       <c r="E36" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B37" s="22">
         <v>46080</v>
       </c>
       <c r="C37" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D37">
         <v>13.64</v>
       </c>
       <c r="E37" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B38" s="22">
         <v>46081</v>
       </c>
       <c r="C38" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D38">
         <v>30</v>
       </c>
       <c r="E38" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B39" s="22">
         <v>46085</v>
       </c>
       <c r="C39" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D39">
         <v>9.2</v>
       </c>
       <c r="E39" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B40" s="22">
         <v>46086</v>
       </c>
       <c r="C40" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D40">
         <v>9.6</v>
       </c>
       <c r="E40" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B41" s="22">
         <v>46087</v>
       </c>
       <c r="C41" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D41">
         <v>8.48</v>
       </c>
       <c r="E41" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B42" s="22">
         <v>46088</v>
       </c>
       <c r="C42" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D42">
         <v>26.72</v>
       </c>
       <c r="E42" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B43" s="22">
         <v>46091</v>
       </c>
       <c r="C43" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D43">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B44" s="22">
         <v>46092</v>
       </c>
       <c r="C44" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D44">
         <v>11.2</v>
       </c>
       <c r="E44" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B45" s="22">
         <v>46093</v>
       </c>
       <c r="C45" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="D45">
         <v>9</v>
       </c>
       <c r="E45" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B46" s="22">
         <v>46094</v>
       </c>
       <c r="C46" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="D46">
         <v>10.8</v>
       </c>
       <c r="E46" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B47" s="22">
         <v>46095</v>
       </c>
       <c r="C47" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D47">
         <v>26.2</v>
       </c>
       <c r="E47" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B48" s="22">
         <v>46098</v>
       </c>
       <c r="C48" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="D48">
         <v>10.8</v>
       </c>
       <c r="E48" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B49" s="22">
         <v>46099</v>
       </c>
       <c r="C49" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D49">
         <v>10</v>
       </c>
       <c r="E49" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B50" s="22">
         <v>46100</v>
       </c>
       <c r="C50" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="D50">
         <v>9.6</v>
       </c>
       <c r="E50" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B51" s="22">
         <v>46101</v>
       </c>
       <c r="C51" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D51">
         <v>11.4</v>
       </c>
       <c r="E51" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B52" s="22">
         <v>46102</v>
       </c>
       <c r="C52" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D52">
         <v>28.2</v>
       </c>
       <c r="E52" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B53" s="22">
         <v>46105</v>
       </c>
       <c r="C53" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="D53">
         <v>8.6</v>
       </c>
       <c r="E53" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B54" s="22">
         <v>46106</v>
       </c>
       <c r="C54" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D54">
         <v>9.2</v>
       </c>
       <c r="E54" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B55" s="22">
         <v>46107</v>
       </c>
       <c r="C55" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="D55">
         <v>8.92</v>
       </c>
       <c r="E55" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B56" s="22">
         <v>46108</v>
       </c>
       <c r="C56" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D56">
         <v>10</v>
       </c>
       <c r="E56" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B57" s="22">
         <v>46109</v>
       </c>
       <c r="C57" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D57">
         <v>25.52</v>
       </c>
       <c r="E57" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B58" s="22">
         <v>46112</v>
       </c>
       <c r="C58" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D58">
         <v>13.2</v>
       </c>
       <c r="E58" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B59" s="22">
         <v>46113</v>
       </c>
       <c r="C59" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="D59">
         <v>9.2</v>
       </c>
       <c r="E59" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B60" s="22">
         <v>46114</v>
       </c>
       <c r="C60" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D60">
         <v>9.24</v>
       </c>
       <c r="E60" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B61" s="22">
         <v>46119</v>
       </c>
       <c r="C61" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="D61">
         <v>10.24</v>
       </c>
       <c r="E61" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B62" s="22">
         <v>46120</v>
       </c>
       <c r="C62" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D62">
         <v>9.28</v>
       </c>
       <c r="E62" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B63" s="22">
         <v>46121</v>
       </c>
       <c r="C63" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D63">
         <v>12.2</v>
       </c>
       <c r="E63" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B64" s="22">
         <v>46122</v>
       </c>
       <c r="C64" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D64">
         <v>9.24</v>
       </c>
       <c r="E64" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B65" s="22">
         <v>46123</v>
       </c>
       <c r="C65" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="D65">
         <v>25.4</v>
       </c>
       <c r="E65" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B66" s="22">
         <v>46126</v>
       </c>
       <c r="C66" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D66">
         <v>14</v>
       </c>
       <c r="E66" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B67" s="22">
         <v>46127</v>
       </c>
       <c r="C67" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D67">
         <v>8.6</v>
       </c>
       <c r="E67" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B68" s="22">
         <v>46128</v>
       </c>
       <c r="C68" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D68">
         <v>8.8</v>
       </c>
       <c r="E68" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B69" s="22">
         <v>46129</v>
       </c>
       <c r="C69" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D69">
         <v>8.8</v>
       </c>
       <c r="E69" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B70" s="22">
         <v>46130</v>
       </c>
       <c r="C70" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="D70">
         <v>25.2</v>
       </c>
       <c r="E70" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B71" s="22">
         <v>46134</v>
       </c>
       <c r="C71" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="D71">
         <v>10.4</v>
       </c>
       <c r="E71" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B72" s="22">
         <v>46135</v>
       </c>
       <c r="C72" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D72">
         <v>8.88</v>
       </c>
       <c r="E72" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B73" s="22">
         <v>46136</v>
       </c>
       <c r="C73" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="D73">
         <v>11</v>
       </c>
       <c r="E73" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B74" s="22">
         <v>46137</v>
       </c>
       <c r="C74" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D74">
         <v>25.2</v>
       </c>
       <c r="E74" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B75" s="22">
         <v>46140</v>
       </c>
       <c r="C75" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="D75">
         <v>12.96</v>
       </c>
       <c r="E75" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B76" s="22">
         <v>46141</v>
       </c>
       <c r="C76" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="D76">
         <v>9.8</v>
       </c>
       <c r="E76" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B77" s="22">
         <v>46142</v>
       </c>
       <c r="C77" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D77">
         <v>10.28</v>
       </c>
       <c r="E77" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B78" s="22">
         <v>46144</v>
       </c>
       <c r="C78" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="D78">
         <v>19.28</v>
       </c>
       <c r="E78" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B79" s="22">
         <v>46147</v>
       </c>
       <c r="C79" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D79">
         <v>7.8</v>
       </c>
       <c r="E79" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="B80" s="22">
         <v>46148</v>
       </c>
       <c r="C80" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D80">
         <v>7.4</v>
       </c>
       <c r="E80" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B81" s="22">
         <v>46149</v>
       </c>
       <c r="C81" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="D81">
         <v>7.8</v>
       </c>
       <c r="E81" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B82" s="22">
         <v>46154</v>
       </c>
       <c r="C82" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D82">
         <v>13.4</v>
       </c>
       <c r="E82" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B83" s="22">
         <v>46155</v>
       </c>
       <c r="C83" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D83">
         <v>9</v>
       </c>
       <c r="E83" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B84" s="22">
         <v>46156</v>
       </c>
       <c r="C84" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="D84">
         <v>8.4</v>
       </c>
       <c r="E84" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B85" s="22">
         <v>46157</v>
       </c>
       <c r="C85" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D85">
         <v>9.2</v>
       </c>
       <c r="E85" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B86" s="22">
         <v>46158</v>
       </c>
       <c r="C86" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D86">
         <v>18</v>
       </c>
       <c r="E86" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B87" s="22">
         <v>46161</v>
       </c>
       <c r="C87" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="D87">
         <v>8</v>
       </c>
       <c r="E87" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B88" s="22">
         <v>46162</v>
       </c>
       <c r="C88" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="D88">
         <v>11.8</v>
       </c>
       <c r="E88" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B89" s="22">
         <v>46163</v>
       </c>
       <c r="C89" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="D89">
         <v>9.2</v>
       </c>
       <c r="E89" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B90" s="22">
         <v>46164</v>
       </c>
       <c r="C90" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D90">
         <v>10.8</v>
       </c>
       <c r="E90" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B91" s="22">
         <v>46165</v>
       </c>
       <c r="C91" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="D91">
         <v>26.08</v>
       </c>
       <c r="E91" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="B92" s="22">
         <v>46168</v>
       </c>
       <c r="C92" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="D92">
         <v>11.8</v>
       </c>
       <c r="E92" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B93" s="22">
         <v>46169</v>
       </c>
       <c r="C93" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="D93">
         <v>9.2</v>
       </c>
       <c r="E93" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B94" s="22">
         <v>46170</v>
       </c>
       <c r="C94" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D94">
         <v>8.8</v>
       </c>
       <c r="E94" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B95" s="22">
         <v>46171</v>
       </c>
       <c r="C95" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D95">
         <v>9.6</v>
       </c>
       <c r="E95" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B96" s="22">
         <v>46172</v>
       </c>
       <c r="C96" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="D96">
         <v>25.48</v>
       </c>
       <c r="E96" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B97" s="22">
         <v>46173</v>
       </c>
       <c r="C97" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D97">
         <v>0.04</v>
       </c>
       <c r="E97" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -11284,16 +11372,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -11307,7 +11395,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F4" s="8">
         <v>1333</v>
@@ -11327,7 +11415,7 @@
         <v>58.999999999999986</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F5" s="8">
         <v>1271.2</v>
@@ -11347,7 +11435,7 @@
         <v>46</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F6" s="8">
         <v>1343.1999999999998</v>
@@ -11367,7 +11455,7 @@
         <v>44</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F7" s="8">
         <v>1193.6000000000001</v>
@@ -11387,7 +11475,7 @@
         <v>47.999999999999986</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F8" s="8">
         <v>1155.2</v>
@@ -11407,7 +11495,7 @@
         <v>127.4</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F9" s="8">
         <v>0</v>
@@ -11427,7 +11515,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F10" s="8">
         <v>0</v>
@@ -11438,14 +11526,14 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="20">
         <v>324.4</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -11456,7 +11544,7 @@
     </row>
     <row r="12" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E12" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -11467,7 +11555,7 @@
     </row>
     <row r="13" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E13" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F13" s="8">
         <v>0</v>
@@ -11478,7 +11566,7 @@
     </row>
     <row r="14" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E14" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F14" s="8">
         <v>0</v>
@@ -11489,7 +11577,7 @@
     </row>
     <row r="15" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E15" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F15" s="8">
         <v>0</v>
@@ -11500,7 +11588,7 @@
     </row>
     <row r="16" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E16" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F16" s="8">
         <v>6296.2</v>

</xml_diff>